<commit_message>
feat: Added source column to the variable excel
</commit_message>
<xml_diff>
--- a/source/bear_attack_model_variables.xlsx
+++ b/source/bear_attack_model_variables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/aminor_ethz_ch/Documents/Master/2026-FS/Participatory Environmental Modelling/PEM_Project/pem_python_test/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="11_18179F0ED376944EE049DC94562D1E7D29755F32" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40E074DA-D59A-4D7D-9143-9EE395D031B7}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="11_18179F0ED376944EE049DC94562D1E7D29755F32" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EF6BDE4-3B89-4315-B565-707C6C5F6685}"/>
   <bookViews>
     <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="107">
   <si>
     <t>Name</t>
   </si>
@@ -226,27 +226,18 @@
     <t>Share of small livestock protected</t>
   </si>
   <si>
-    <t>Fraction of small livestock units (0-1) covered by the protective measure (e.g., behind an electric fence or in a guarded pen). The actual protected count is this share times N_SL.</t>
-  </si>
-  <si>
     <t>s_prot_SL</t>
   </si>
   <si>
     <t>Share of large livestock protected</t>
   </si>
   <si>
-    <t>Fraction of large livestock units (0-1) covered by the protective measure.</t>
-  </si>
-  <si>
     <t>s_prot_LL</t>
   </si>
   <si>
     <t>Share of agriculture protected</t>
   </si>
   <si>
-    <t>Fraction of agricultural units (0-1) covered by the protective measure (e.g., beehives behind a bear-proof fence).</t>
-  </si>
-  <si>
     <t>s_prot_Ag</t>
   </si>
   <si>
@@ -320,13 +311,43 @@
   </si>
   <si>
     <t>Need - ask experts</t>
+  </si>
+  <si>
+    <t>Natura Protetta Orso Marsicano (2024)</t>
+  </si>
+  <si>
+    <t>Needs to be asked - Interviews with experts</t>
+  </si>
+  <si>
+    <t>Calculated</t>
+  </si>
+  <si>
+    <t>Baseline comes from Salviamo l'orso (2026), works as a slider.</t>
+  </si>
+  <si>
+    <t>Percentage of protected small livestock units (e.g., behind an electric fence or in a guarded pen). The actual protected count is this share times N_SL.</t>
+  </si>
+  <si>
+    <t>Percentage of protected large livestock units (e.g., behind an electric fence or in a guarded pen). The actual protected count is this share times N_SL.</t>
+  </si>
+  <si>
+    <t>Percentage of protected agricultrue units (e.g., behind an electric fence or in a guarded pen). The actual protected count is this share times N_SL.</t>
+  </si>
+  <si>
+    <t>Either baseline or assumption - needs slided</t>
+  </si>
+  <si>
+    <t>Needs to be asked to Berenice or Paula</t>
+  </si>
+  <si>
+    <t>Slider</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -350,6 +371,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -440,7 +472,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -483,6 +515,36 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -811,7 +873,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
@@ -828,7 +890,7 @@
         <v>0.6</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
@@ -845,28 +907,28 @@
         <v>0.85</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="5" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D4" s="5">
         <v>2200</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="16" t="s">
         <v>11</v>
       </c>
       <c r="C5" s="11" t="s">
@@ -877,10 +939,10 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="16" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -903,6 +965,9 @@
       <c r="D7" s="9">
         <v>0.85</v>
       </c>
+      <c r="E7" s="18" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="8" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
@@ -917,6 +982,9 @@
       <c r="D8" s="9">
         <v>0.35</v>
       </c>
+      <c r="E8" s="18" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="9" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
@@ -931,6 +999,9 @@
       <c r="D9" s="9">
         <v>0.65</v>
       </c>
+      <c r="E9" s="18" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="10" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
@@ -945,6 +1016,9 @@
       <c r="D10" s="6">
         <v>0.66</v>
       </c>
+      <c r="E10" s="17" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="11" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
@@ -959,6 +1033,9 @@
       <c r="D11" s="6">
         <v>0.1</v>
       </c>
+      <c r="E11" s="17" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="12" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
@@ -973,6 +1050,9 @@
       <c r="D12" s="6">
         <v>0.24</v>
       </c>
+      <c r="E12" s="17" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="13" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="7" t="s">
@@ -987,6 +1067,9 @@
       <c r="D13" s="8">
         <v>0.85</v>
       </c>
+      <c r="E13" s="8" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="14" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="7" t="s">
@@ -1001,6 +1084,9 @@
       <c r="D14" s="8">
         <v>0.15</v>
       </c>
+      <c r="E14" s="8" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="15" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
@@ -1015,6 +1101,9 @@
       <c r="D15" s="5">
         <v>15000</v>
       </c>
+      <c r="E15" s="20" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="16" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="5" t="s">
@@ -1029,8 +1118,11 @@
       <c r="D16" s="5">
         <v>2500</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E16" s="20" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="5" t="s">
         <v>46</v>
       </c>
@@ -1043,8 +1135,11 @@
       <c r="D17" s="5">
         <v>2000</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E17" s="20" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
         <v>49</v>
       </c>
@@ -1057,8 +1152,11 @@
       <c r="D18" s="3">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E18" s="18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
         <v>52</v>
       </c>
@@ -1071,8 +1169,11 @@
       <c r="D19" s="3">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E19" s="18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
         <v>55</v>
       </c>
@@ -1085,8 +1186,11 @@
       <c r="D20" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E20" s="18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>58</v>
       </c>
@@ -1099,8 +1203,11 @@
       <c r="D21" s="4">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E21" s="19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
         <v>61</v>
       </c>
@@ -1113,8 +1220,11 @@
       <c r="D22" s="4">
         <v>800</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E22" s="15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
         <v>64</v>
       </c>
@@ -1127,131 +1237,161 @@
       <c r="D23" s="4">
         <v>600</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E23" s="15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="D24" s="12">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E24" s="22" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="D25" s="12">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E25" s="22" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>103</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D26" s="12">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E26" s="22" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D27" s="5">
         <v>20</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E27" s="23" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D28" s="5">
         <v>80</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E28" s="23" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D29" s="5">
         <v>80</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E29" s="23" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D30" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E30" s="19" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D31" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="27" x14ac:dyDescent="0.45">
+      <c r="E31" s="24" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="27" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D32" s="2">
         <v>12</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: put correct allied NGO name, Rewilding Apennines, instead of Salviamo l'orso
</commit_message>
<xml_diff>
--- a/source/bear_attack_model_variables.xlsx
+++ b/source/bear_attack_model_variables.xlsx
@@ -8,19 +8,38 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/aminor_ethz_ch/Documents/Master/2026-FS/Participatory Environmental Modelling/PEM_Project/pem_python_test/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_ED0446E7D443CC9E621180974728DE3FF3E801AF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BA76346-659D-41B2-9961-D98A7A3B1193}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="11_ED0446E7D443CC9E621180974728DE3FF3E801AF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B1F72BD-A3CE-44C7-96DF-BC06E6956F90}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Model Variables" sheetId="1" r:id="rId1"/>
+    <sheet name="default_general" sheetId="1" r:id="rId1"/>
+    <sheet name="default_mun1" sheetId="6" r:id="rId2"/>
+    <sheet name="default_mun2" sheetId="4" r:id="rId3"/>
+    <sheet name="default_mun3" sheetId="5" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="105">
   <si>
     <t>Name</t>
   </si>
@@ -37,6 +56,9 @@
     <t>Source</t>
   </si>
   <si>
+    <t>Average incursions per year and bear</t>
+  </si>
+  <si>
     <t>Estimated number of bear incursions per year in the broader area surrounding the property - a baseline pressure metric used to scale the attack rate.</t>
   </si>
   <si>
@@ -332,16 +354,13 @@
   </si>
   <si>
     <t>Slider</t>
-  </si>
-  <si>
-    <t>Average incursions per year and bear</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -377,8 +396,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -426,8 +450,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -461,12 +491,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -537,7 +595,72 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="7" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="7" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="7" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -870,530 +993,2274 @@
     </row>
     <row r="2" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>104</v>
+        <v>5</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="5">
         <v>350</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" s="5">
         <v>5</v>
       </c>
-      <c r="E3" s="24" t="s">
-        <v>7</v>
+      <c r="E3" s="5" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" s="10">
         <v>1</v>
       </c>
+      <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="9">
         <v>0.85</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="9">
         <v>0.35</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D7" s="9">
         <v>0.65</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D8" s="6">
         <v>0.66</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D9" s="6">
         <v>0.1</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D10" s="6">
         <v>0.24</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D11" s="8">
         <v>0.85</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D12" s="8">
         <v>0.15</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D13" s="5">
         <v>15000</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D14" s="5">
         <v>2500</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D15" s="5">
         <v>2000</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D16" s="3">
         <v>10</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D17" s="3">
         <v>2</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D18" s="3">
         <v>6</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D19" s="4">
         <v>50</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D20" s="4">
         <v>800</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D21" s="4">
         <v>600</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D22" s="11">
         <v>0.6</v>
       </c>
       <c r="E22" s="21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D23" s="11">
         <v>0.25</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D24" s="11">
         <v>0.2</v>
       </c>
       <c r="E24" s="21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D25" s="5">
         <v>20</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D26" s="5">
         <v>80</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D27" s="5">
         <v>80</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D28" s="4">
         <v>5</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D29" s="4">
         <v>20</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D30" s="4">
         <v>5</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D31" s="2">
         <v>10</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>100</v>
+      <c r="A32" s="20" t="s">
+        <v>101</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D32" s="2">
         <v>12</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" ht="27" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08EB3E2D-826E-4F8D-9613-E45946C2E63B}">
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="48" customWidth="1"/>
+    <col min="2" max="2" width="80" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="96.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="27">
+        <v>5</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="30">
+        <v>0.85</v>
+      </c>
+      <c r="E3" s="43" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="30">
+        <v>0.15</v>
+      </c>
+      <c r="E4" s="43" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="27">
+        <v>15000</v>
+      </c>
+      <c r="E5" s="44" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="27">
+        <v>2500</v>
+      </c>
+      <c r="E6" s="44" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="27">
+        <v>2000</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="35">
+        <v>0.6</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="35">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="E10" s="36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="37" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="38">
+        <f>_xlfn.XLOOKUP(A11,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>350</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="40" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="38">
+        <f>_xlfn.XLOOKUP(A12,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>1</v>
+      </c>
+      <c r="E12" s="40"/>
+    </row>
+    <row r="13" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="45">
+        <f>_xlfn.XLOOKUP(A13,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.85</v>
+      </c>
+      <c r="E13" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="45">
+        <f>_xlfn.XLOOKUP(A14,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.35</v>
+      </c>
+      <c r="E14" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="45">
+        <f>_xlfn.XLOOKUP(A15,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.65</v>
+      </c>
+      <c r="E15" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="45">
+        <f>_xlfn.XLOOKUP(A16,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.66</v>
+      </c>
+      <c r="E16" s="40" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="45">
+        <f>_xlfn.XLOOKUP(A17,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="40" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="45">
+        <f>_xlfn.XLOOKUP(A18,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.24</v>
+      </c>
+      <c r="E18" s="40" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="38">
+        <f>_xlfn.XLOOKUP(A19,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>10</v>
+      </c>
+      <c r="E19" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="38">
+        <f>_xlfn.XLOOKUP(A20,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>2</v>
+      </c>
+      <c r="E20" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="C21" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="38">
+        <f>_xlfn.XLOOKUP(A21,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>6</v>
+      </c>
+      <c r="E21" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A22" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" s="38">
+        <f>_xlfn.XLOOKUP(A22,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>50</v>
+      </c>
+      <c r="E22" s="41" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A23" s="37" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="38">
+        <f>_xlfn.XLOOKUP(A23,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>800</v>
+      </c>
+      <c r="E23" s="39" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A24" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="D24" s="38">
+        <f>_xlfn.XLOOKUP(A24,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>600</v>
+      </c>
+      <c r="E24" s="39" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" s="38">
+        <f>_xlfn.XLOOKUP(A25,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>20</v>
+      </c>
+      <c r="E25" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="38">
+        <f>_xlfn.XLOOKUP(A26,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>80</v>
+      </c>
+      <c r="E26" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="D27" s="38">
+        <f>_xlfn.XLOOKUP(A27,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>80</v>
+      </c>
+      <c r="E27" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="38">
+        <f>_xlfn.XLOOKUP(A28,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>5</v>
+      </c>
+      <c r="E28" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="38">
+        <f>_xlfn.XLOOKUP(A29,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>20</v>
+      </c>
+      <c r="E29" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30" s="38">
+        <f>_xlfn.XLOOKUP(A30,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>5</v>
+      </c>
+      <c r="E30" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="38">
+        <f>_xlfn.XLOOKUP(A31,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>10</v>
+      </c>
+      <c r="E31" s="39" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="B32" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="D32" s="38">
+        <f>_xlfn.XLOOKUP(A32,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>12</v>
+      </c>
+      <c r="E32" s="39" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E640EAA-98EC-40F6-817C-E7CACD5BDB7F}">
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="48" customWidth="1"/>
+    <col min="2" max="2" width="80" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="89.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="27">
+        <v>5</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="30">
+        <v>0.85</v>
+      </c>
+      <c r="E3" s="43" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="30">
+        <v>0.15</v>
+      </c>
+      <c r="E4" s="43" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="27">
+        <v>15000</v>
+      </c>
+      <c r="E5" s="44" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="27">
+        <v>2500</v>
+      </c>
+      <c r="E6" s="44" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="27">
+        <v>2000</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="35">
+        <v>0.6</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="35">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="E10" s="36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="37" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="38">
+        <f>_xlfn.XLOOKUP(A11,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>350</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="40" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="38">
+        <f>_xlfn.XLOOKUP(A12,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>1</v>
+      </c>
+      <c r="E12" s="40"/>
+    </row>
+    <row r="13" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="45">
+        <f>_xlfn.XLOOKUP(A13,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.85</v>
+      </c>
+      <c r="E13" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="45">
+        <f>_xlfn.XLOOKUP(A14,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.35</v>
+      </c>
+      <c r="E14" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="45">
+        <f>_xlfn.XLOOKUP(A15,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.65</v>
+      </c>
+      <c r="E15" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="45">
+        <f>_xlfn.XLOOKUP(A16,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.66</v>
+      </c>
+      <c r="E16" s="40" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="45">
+        <f>_xlfn.XLOOKUP(A17,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="40" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="45">
+        <f>_xlfn.XLOOKUP(A18,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.24</v>
+      </c>
+      <c r="E18" s="40" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="38">
+        <f>_xlfn.XLOOKUP(A19,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>10</v>
+      </c>
+      <c r="E19" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="38">
+        <f>_xlfn.XLOOKUP(A20,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>2</v>
+      </c>
+      <c r="E20" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="C21" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="38">
+        <f>_xlfn.XLOOKUP(A21,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>6</v>
+      </c>
+      <c r="E21" s="40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A22" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" s="38">
+        <f>_xlfn.XLOOKUP(A22,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>50</v>
+      </c>
+      <c r="E22" s="41" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A23" s="37" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="38">
+        <f>_xlfn.XLOOKUP(A23,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>800</v>
+      </c>
+      <c r="E23" s="39" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A24" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="D24" s="38">
+        <f>_xlfn.XLOOKUP(A24,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>600</v>
+      </c>
+      <c r="E24" s="39" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" s="38">
+        <f>_xlfn.XLOOKUP(A25,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>20</v>
+      </c>
+      <c r="E25" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="38">
+        <f>_xlfn.XLOOKUP(A26,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>80</v>
+      </c>
+      <c r="E26" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="D27" s="38">
+        <f>_xlfn.XLOOKUP(A27,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>80</v>
+      </c>
+      <c r="E27" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="38">
+        <f>_xlfn.XLOOKUP(A28,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>5</v>
+      </c>
+      <c r="E28" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="38">
+        <f>_xlfn.XLOOKUP(A29,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>20</v>
+      </c>
+      <c r="E29" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30" s="38">
+        <f>_xlfn.XLOOKUP(A30,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>5</v>
+      </c>
+      <c r="E30" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="38">
+        <f>_xlfn.XLOOKUP(A31,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>10</v>
+      </c>
+      <c r="E31" s="39" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="B32" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="D32" s="38">
+        <f>_xlfn.XLOOKUP(A32,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>12</v>
+      </c>
+      <c r="E32" s="39" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5405BA5-D6DA-4CE3-8907-A1E7184D4C76}">
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="48" customWidth="1"/>
+    <col min="2" max="2" width="80" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="105.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="27">
+        <v>5</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="30">
+        <v>0.85</v>
+      </c>
+      <c r="E3" s="31" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="30">
+        <v>0.15</v>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="27">
+        <v>15000</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="27">
+        <v>2500</v>
+      </c>
+      <c r="E6" s="32" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="27">
+        <v>2000</v>
+      </c>
+      <c r="E7" s="32" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="35">
+        <v>0.6</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="35">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="35">
+        <v>0.2</v>
+      </c>
+      <c r="E10" s="36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="37" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="24">
+        <f>_xlfn.XLOOKUP(A11,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>350</v>
+      </c>
+      <c r="E11" s="39" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="40" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="24">
+        <f>_xlfn.XLOOKUP(A12,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>1</v>
+      </c>
+      <c r="E12" s="41"/>
+    </row>
+    <row r="13" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="42">
+        <f>_xlfn.XLOOKUP(A13,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.85</v>
+      </c>
+      <c r="E13" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="42">
+        <f>_xlfn.XLOOKUP(A14,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.35</v>
+      </c>
+      <c r="E14" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="42">
+        <f>_xlfn.XLOOKUP(A15,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.65</v>
+      </c>
+      <c r="E15" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="42">
+        <f>_xlfn.XLOOKUP(A16,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.66</v>
+      </c>
+      <c r="E16" s="41" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="42">
+        <f>_xlfn.XLOOKUP(A17,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="41" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="42">
+        <f>_xlfn.XLOOKUP(A18,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>0.24</v>
+      </c>
+      <c r="E18" s="41" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="24">
+        <f>_xlfn.XLOOKUP(A19,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>10</v>
+      </c>
+      <c r="E19" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="24">
+        <f>_xlfn.XLOOKUP(A20,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>2</v>
+      </c>
+      <c r="E20" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="C21" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="24">
+        <f>_xlfn.XLOOKUP(A21,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>6</v>
+      </c>
+      <c r="E21" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A22" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" s="24">
+        <f>_xlfn.XLOOKUP(A22,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>50</v>
+      </c>
+      <c r="E22" s="41" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A23" s="37" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="24">
+        <f>_xlfn.XLOOKUP(A23,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>800</v>
+      </c>
+      <c r="E23" s="39" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A24" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="D24" s="24">
+        <f>_xlfn.XLOOKUP(A24,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>600</v>
+      </c>
+      <c r="E24" s="39" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" s="24">
+        <f>_xlfn.XLOOKUP(A25,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>20</v>
+      </c>
+      <c r="E25" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="24">
+        <f>_xlfn.XLOOKUP(A26,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>80</v>
+      </c>
+      <c r="E26" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="D27" s="24">
+        <f>_xlfn.XLOOKUP(A27,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>80</v>
+      </c>
+      <c r="E27" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="24">
+        <f>_xlfn.XLOOKUP(A28,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>5</v>
+      </c>
+      <c r="E28" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="24">
+        <f>_xlfn.XLOOKUP(A29,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>20</v>
+      </c>
+      <c r="E29" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30" s="24">
+        <f>_xlfn.XLOOKUP(A30,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>5</v>
+      </c>
+      <c r="E30" s="41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="24">
+        <f>_xlfn.XLOOKUP(A31,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>10</v>
+      </c>
+      <c r="E31" s="39" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="B32" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="D32" s="24">
+        <f>_xlfn.XLOOKUP(A32,default_general!$A$2:$A$32,default_general!$D$2:$D$32,"Error",0)</f>
+        <v>12</v>
+      </c>
+      <c r="E32" s="39" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>